<commit_message>
feat(schema): add phase screening and the legal sources of lung-cancer screening
Prepares the screening episode (LDCT lung-cancer screening under LuKrFrühErkV and
G-BA KFE-RL) as a fifth phase, following the eight steps of docs/howto-add-element.md §D:

- schema: phase enum and ID pattern gain `screening`; the guideline_references source
  enum gains `LuKrFrühErkV` and `G-BA KFE-RL` (legal norms, no recommendation grade),
  documented in the field description.
- elements/screening/ with a README (empty until the first elements are adopted).
- build-catalog.py phase list, _elicitation.py phase dropdown, FSH generator
  (PhasesCS, GuidelineSourceCS), issue form, CODEOWNERS; regenerated elicitation
  template and phases overview.

Minor schema change: all existing YAMLs stay valid.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/datenelement-erhebung.xlsx
+++ b/templates/datenelement-erhebung.xlsx
@@ -2097,7 +2097,7 @@
       <formula1>=Codelisten!$B$2:$B$18</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E62" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Ungültige Eingabe" error="Bitte aus der Liste wählen." type="list" errorStyle="stop">
-      <formula1>=Codelisten!$A$2:$A$6</formula1>
+      <formula1>=Codelisten!$A$2:$A$7</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Codelisten!$C$2:$C$5</formula1>
@@ -2127,7 +2127,7 @@
       <formula1>=Codelisten!$H$2:$H$19</formula1>
     </dataValidation>
     <dataValidation sqref="Q2:Q62" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Ungültige Eingabe" error="Bitte aus der Liste wählen." type="list" errorStyle="stop">
-      <formula1>=Codelisten!$I$2:$I$12</formula1>
+      <formula1>=Codelisten!$I$2:$I$14</formula1>
     </dataValidation>
     <dataValidation sqref="S2:S62" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Ungültige Eingabe" error="Bitte aus der Liste wählen." type="list" errorStyle="stop">
       <formula1>=Codelisten!$J$2:$J$7</formula1>
@@ -4057,7 +4057,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Onkologische Nachsorge (kurativ behandelt)</t>
+          <t>Krebsfrüherkennung / LDCT-Screening</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4154,7 +4154,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Verlaufsbeobachtung / Surveillance (unter Systemtherapie)</t>
+          <t>Onkologische Nachsorge (kurativ behandelt)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -4251,7 +4251,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Palliativversorgung</t>
+          <t>Verlaufsbeobachtung / Surveillance (unter Systemtherapie)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4343,7 +4343,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Hausärztliche Versorgung / sektorenübergreifende Basisdaten</t>
+          <t>Palliativversorgung</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -4435,71 +4435,76 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Hausärztliche Versorgung / sektorenübergreifende Basisdaten</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Kontakt/Visite</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Datum + Uhrzeit</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>kbv-mio</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Onkopedia SCLC</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Statement</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Labor-/Pathologie-IS (LIS)</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>übermittelt / ausgetauscht</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>icf</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>cm</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Tumorboard / MDT</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>Andere / neue Phase (rechts benennen)</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Kontakt/Visite</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Datum + Uhrzeit</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>kbv-mio</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Onkopedia SCLC</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Statement</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Labor-/Pathologie-IS (LIS)</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>übermittelt / ausgetauscht</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>icf</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>cm</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>Tumorboard / MDT</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
       <c r="B7" t="inlineStr">
         <is>
           <t>Versorgungsplanung</t>
@@ -4782,7 +4787,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>andere</t>
+          <t>LuKrFrühErkV</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -4817,6 +4822,11 @@
           <t>omop-cdm</t>
         </is>
       </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>G-BA KFE-RL</t>
+        </is>
+      </c>
       <c r="O13" t="inlineStr">
         <is>
           <t>local-no-standard-binding</t>
@@ -4837,6 +4847,11 @@
       <c r="H14" t="inlineStr">
         <is>
           <t>cdisc-sdtm</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>andere</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">

</xml_diff>